<commit_message>
feat: implement dark mode support for maps and UI components
- Added useDarkMode hook to manage dark mode state.
- Updated LeafletMap, HubPickerMap, and RouteMap components to use dark mode tiles and styles.
- Enhanced RouteMap to display additional delivery details including meals and notes.
- Introduced PNG export functionality for the shipping table.
- Refactored sidebar and shipping table components for improved UI and accessibility.
- Added new data files for order day addresses and updated existing test data.
</commit_message>
<xml_diff>
--- a/data/test/notes.xlsx
+++ b/data/test/notes.xlsx
@@ -397,10 +397,45 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
-  <sheetData/>
+  <dimension ref="A1:E2"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>id</v>
+      </c>
+      <c r="B1" t="str">
+        <v>weekLabel</v>
+      </c>
+      <c r="C1" t="str">
+        <v>customerId</v>
+      </c>
+      <c r="D1" t="str">
+        <v>day</v>
+      </c>
+      <c r="E1" t="str">
+        <v>note</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>2026-W20-0901000005-1</v>
+      </c>
+      <c r="B2" t="str">
+        <v>2026-W20</v>
+      </c>
+      <c r="C2" t="str">
+        <v>0901000005</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+      <c r="E2" t="str">
+        <v>lấy nhiều thịt nướng</v>
+      </c>
+    </row>
+  </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>